<commit_message>
Added Repeat Offering Dialogue, fixed stone gate hint
</commit_message>
<xml_diff>
--- a/DesignDocs/bound_spirit_dialogues.xlsx
+++ b/DesignDocs/bound_spirit_dialogues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR\Unity Projects\Class Assignments\CS 425\CS425-Senior-Project\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EFE8C8B-553C-4261-B46A-039E64E5DE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD6F3C8-011D-4180-A19A-A074598A9A42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7380" yWindow="1524" windowWidth="18432" windowHeight="10680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6144" yWindow="516" windowWidth="18432" windowHeight="12540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="204">
   <si>
     <t>Bound Spirit Dialogue Workbook</t>
   </si>
@@ -590,6 +590,54 @@
   </si>
   <si>
     <t>Gentle Ghost</t>
+  </si>
+  <si>
+    <t>Ghost1NeedRepeat.asset</t>
+  </si>
+  <si>
+    <t>Ghost1NeedRepeat</t>
+  </si>
+  <si>
+    <t>Ghost2NeedRepeat.asset</t>
+  </si>
+  <si>
+    <t>Ghost2NeedRepeat</t>
+  </si>
+  <si>
+    <t>Did you find the words I never finished?</t>
+  </si>
+  <si>
+    <t>Ghost3NeedRepeat.asset</t>
+  </si>
+  <si>
+    <t>Ghost3NeedRepeat</t>
+  </si>
+  <si>
+    <t>Did you find what once carried that sweet scent?</t>
+  </si>
+  <si>
+    <t>What happened to me? How did I die?</t>
+  </si>
+  <si>
+    <t>The stone beneath the gate is worn smooth by time.</t>
+  </si>
+  <si>
+    <t>Three faint markings are carved into its surface.</t>
+  </si>
+  <si>
+    <t>Someone scratched a message below them:</t>
+  </si>
+  <si>
+    <t>“Three memories linger in this graveyard. Return what was lost… and the path will open.”</t>
+  </si>
+  <si>
+    <t>The carving beneath the gate is still visible.</t>
+  </si>
+  <si>
+    <t>“Three memories… Return what was lost, and the path will open.”</t>
+  </si>
+  <si>
+    <t>There\u2019s some sort of seal on the gate. Maybe there's a clue nearby...</t>
   </si>
 </sst>
 </file>
@@ -1104,7 +1152,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
@@ -1112,7 +1160,7 @@
     <col min="3" max="3" width="35.21875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="72" customWidth="1"/>
+    <col min="6" max="6" width="92.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
     <col min="8" max="8" width="24" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
@@ -1224,24 +1272,12 @@
       <c r="J4" s="6"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="6">
-        <v>0</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>119</v>
-      </c>
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
@@ -1258,13 +1294,13 @@
         <v>39</v>
       </c>
       <c r="D6" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>40</v>
+      <c r="F6" t="s">
+        <v>197</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -1282,13 +1318,13 @@
         <v>39</v>
       </c>
       <c r="D7" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>42</v>
+      <c r="F7" t="s">
+        <v>198</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -1297,22 +1333,22 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="D8" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>129</v>
+        <v>41</v>
+      </c>
+      <c r="F8" t="s">
+        <v>199</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -1321,22 +1357,22 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="D9" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>71</v>
+      <c r="F9" t="s">
+        <v>200</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
@@ -1345,22 +1381,22 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="D10" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>41</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>72</v>
+        <v>201</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
@@ -1369,22 +1405,22 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="D11" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>41</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>73</v>
+        <v>202</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
@@ -1392,24 +1428,12 @@
       <c r="J11" s="6"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D12" s="6">
-        <v>4</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>74</v>
-      </c>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
@@ -1426,13 +1450,13 @@
         <v>68</v>
       </c>
       <c r="D13" s="6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>75</v>
+        <v>129</v>
       </c>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
@@ -1450,13 +1474,13 @@
         <v>68</v>
       </c>
       <c r="D14" s="6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>41</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
@@ -1465,22 +1489,22 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>97</v>
+        <v>67</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>130</v>
+        <v>68</v>
       </c>
       <c r="D15" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>41</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
@@ -1488,12 +1512,24 @@
       <c r="J15" s="6"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+      <c r="A16" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="6">
+        <v>3</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>73</v>
+      </c>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
@@ -1501,22 +1537,22 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="D17" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>187</v>
+        <v>41</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>46</v>
+        <v>196</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
@@ -1525,22 +1561,22 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="D18" s="6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>187</v>
+        <v>41</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>47</v>
+        <v>75</v>
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
@@ -1549,22 +1585,22 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="D19" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="F19" t="s">
-        <v>178</v>
+        <v>41</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>76</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
@@ -1573,22 +1609,22 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
-        <v>43</v>
+        <v>97</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>44</v>
+        <v>130</v>
       </c>
       <c r="D20" s="6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="F20" t="s">
-        <v>179</v>
+        <v>41</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>99</v>
       </c>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
@@ -1596,24 +1632,12 @@
       <c r="J20" s="6"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D21" s="6">
-        <v>4</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="F21" t="s">
-        <v>177</v>
-      </c>
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
@@ -1621,13 +1645,13 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D22" s="6">
         <v>0</v>
@@ -1636,7 +1660,7 @@
         <v>187</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
@@ -1645,13 +1669,13 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D23" s="6">
         <v>1</v>
@@ -1660,7 +1684,7 @@
         <v>187</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
@@ -1669,13 +1693,13 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D24" s="6">
         <v>2</v>
@@ -1683,8 +1707,8 @@
       <c r="E24" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>54</v>
+      <c r="F24" t="s">
+        <v>178</v>
       </c>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
@@ -1693,22 +1717,22 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D25" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>57</v>
+      <c r="F25" t="s">
+        <v>179</v>
       </c>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
@@ -1717,22 +1741,22 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D26" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>186</v>
+      <c r="F26" t="s">
+        <v>177</v>
       </c>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
@@ -1741,22 +1765,22 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
-        <v>55</v>
+        <v>188</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>56</v>
+        <v>189</v>
       </c>
       <c r="D27" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>187</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>59</v>
+        <v>195</v>
       </c>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
@@ -1765,22 +1789,22 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D28" s="6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>187</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>185</v>
+        <v>52</v>
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
@@ -1789,22 +1813,22 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D29" s="6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>187</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
@@ -1813,22 +1837,22 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
-        <v>180</v>
+        <v>50</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>181</v>
+        <v>51</v>
       </c>
       <c r="D30" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="F30" t="s">
-        <v>182</v>
+      <c r="F30" s="6" t="s">
+        <v>54</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
@@ -1837,51 +1861,71 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
-        <v>180</v>
+        <v>55</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>181</v>
+        <v>56</v>
       </c>
       <c r="D31" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="F31" t="s">
-        <v>183</v>
-      </c>
+      <c r="F31" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
-        <v>180</v>
+        <v>55</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>181</v>
+        <v>56</v>
       </c>
       <c r="D32" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="F32" t="s">
-        <v>184</v>
-      </c>
+      <c r="F32" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="6"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A33" s="6"/>
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
+      <c r="A33" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D33" s="6">
+        <v>2</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
       <c r="I33" s="6"/>
@@ -1889,22 +1933,22 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>134</v>
+        <v>56</v>
       </c>
       <c r="D34" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="F34" t="s">
-        <v>143</v>
+        <v>187</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>185</v>
       </c>
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
@@ -1913,22 +1957,22 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>134</v>
+        <v>56</v>
       </c>
       <c r="D35" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="F35" t="s">
-        <v>144</v>
+        <v>187</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>60</v>
       </c>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
@@ -1937,22 +1981,22 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
-        <v>131</v>
+        <v>180</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>134</v>
+        <v>181</v>
       </c>
       <c r="D36" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>137</v>
+        <v>187</v>
       </c>
       <c r="F36" t="s">
-        <v>145</v>
+        <v>182</v>
       </c>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
@@ -1961,71 +2005,51 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
-        <v>131</v>
+        <v>180</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>134</v>
+        <v>181</v>
       </c>
       <c r="D37" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>137</v>
+        <v>187</v>
       </c>
       <c r="F37" t="s">
-        <v>147</v>
-      </c>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
+        <v>183</v>
+      </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
-        <v>131</v>
+        <v>180</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>134</v>
+        <v>181</v>
       </c>
       <c r="D38" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>137</v>
+        <v>187</v>
       </c>
       <c r="F38" t="s">
-        <v>146</v>
-      </c>
-      <c r="G38" s="6"/>
-      <c r="H38" s="6"/>
-      <c r="I38" s="6"/>
-      <c r="J38" s="6"/>
+        <v>184</v>
+      </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A39" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="D39" s="6">
-        <v>0</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="F39" t="s">
-        <v>138</v>
-      </c>
+      <c r="A39" s="6"/>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
       <c r="I39" s="6"/>
@@ -2033,22 +2057,22 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D40" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>137</v>
       </c>
       <c r="F40" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
@@ -2057,22 +2081,22 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D41" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>137</v>
       </c>
       <c r="F41" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
@@ -2081,22 +2105,22 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D42" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>137</v>
       </c>
       <c r="F42" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
@@ -2105,22 +2129,22 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D43" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>137</v>
       </c>
       <c r="F43" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
@@ -2129,22 +2153,22 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D44" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>137</v>
       </c>
       <c r="F44" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
@@ -2153,22 +2177,22 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
-        <v>133</v>
+        <v>190</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>136</v>
+        <v>191</v>
       </c>
       <c r="D45" s="6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>137</v>
       </c>
       <c r="F45" t="s">
-        <v>152</v>
+        <v>192</v>
       </c>
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
@@ -2177,13 +2201,13 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="D46" s="6">
         <v>0</v>
@@ -2192,7 +2216,7 @@
         <v>137</v>
       </c>
       <c r="F46" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
@@ -2201,13 +2225,13 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="D47" s="6">
         <v>1</v>
@@ -2216,18 +2240,22 @@
         <v>137</v>
       </c>
       <c r="F47" t="s">
-        <v>149</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="G47" s="6"/>
+      <c r="H47" s="6"/>
+      <c r="I47" s="6"/>
+      <c r="J47" s="6"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="D48" s="6">
         <v>2</v>
@@ -2236,27 +2264,55 @@
         <v>137</v>
       </c>
       <c r="F48" t="s">
-        <v>150</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="G48" s="6"/>
+      <c r="H48" s="6"/>
+      <c r="I48" s="6"/>
+      <c r="J48" s="6"/>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D49" s="6">
+        <v>0</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F49" t="s">
+        <v>151</v>
+      </c>
+      <c r="G49" s="6"/>
+      <c r="H49" s="6"/>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>172</v>
+        <v>136</v>
       </c>
       <c r="D50" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="F50" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="G50" s="6"/>
       <c r="H50" s="6"/>
@@ -2265,22 +2321,22 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>172</v>
+        <v>136</v>
       </c>
       <c r="D51" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="F51" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G51" s="6"/>
       <c r="H51" s="6"/>
@@ -2289,22 +2345,22 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>172</v>
+        <v>136</v>
       </c>
       <c r="D52" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="F52" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="G52" s="6"/>
       <c r="H52" s="6"/>
@@ -2313,22 +2369,22 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>172</v>
+        <v>141</v>
       </c>
       <c r="D53" s="6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="F53" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
@@ -2337,85 +2393,53 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>172</v>
+        <v>141</v>
       </c>
       <c r="D54" s="6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="F54" t="s">
-        <v>161</v>
-      </c>
-      <c r="G54" s="6"/>
-      <c r="H54" s="6"/>
-      <c r="I54" s="6"/>
-      <c r="J54" s="6"/>
+        <v>149</v>
+      </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
-        <v>169</v>
+        <v>140</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>173</v>
+        <v>141</v>
       </c>
       <c r="D55" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="F55" t="s">
-        <v>167</v>
-      </c>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
-      <c r="I55" s="6"/>
-      <c r="J55" s="6"/>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A56" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="B56" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D56" s="6">
-        <v>1</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="F56" t="s">
-        <v>168</v>
-      </c>
-      <c r="G56" s="6"/>
-      <c r="H56" s="6"/>
-      <c r="I56" s="6"/>
-      <c r="J56" s="6"/>
+        <v>150</v>
+      </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D57" s="6">
         <v>0</v>
@@ -2424,7 +2448,7 @@
         <v>157</v>
       </c>
       <c r="F57" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
@@ -2433,13 +2457,13 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="6" t="s">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D58" s="6">
         <v>1</v>
@@ -2448,7 +2472,7 @@
         <v>157</v>
       </c>
       <c r="F58" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="G58" s="6"/>
       <c r="H58" s="6"/>
@@ -2457,13 +2481,13 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D59" s="6">
         <v>2</v>
@@ -2472,7 +2496,7 @@
         <v>157</v>
       </c>
       <c r="F59" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="G59" s="6"/>
       <c r="H59" s="6"/>
@@ -2481,13 +2505,13 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="s">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D60" s="6">
         <v>3</v>
@@ -2496,7 +2520,7 @@
         <v>157</v>
       </c>
       <c r="F60" t="s">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="G60" s="6"/>
       <c r="H60" s="6"/>
@@ -2505,22 +2529,22 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
-        <v>171</v>
+        <v>142</v>
       </c>
       <c r="B61" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D61" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>157</v>
       </c>
       <c r="F61" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G61" s="6"/>
       <c r="H61" s="6"/>
@@ -2529,49 +2553,70 @@
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="6" t="s">
-        <v>171</v>
+        <v>193</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="D62" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>157</v>
       </c>
       <c r="F62" t="s">
-        <v>163</v>
-      </c>
+        <v>195</v>
+      </c>
+      <c r="G62" s="6"/>
+      <c r="H62" s="6"/>
+      <c r="I62" s="6"/>
+      <c r="J62" s="6"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A63" s="6"/>
-      <c r="B63" s="6"/>
-      <c r="C63" s="6"/>
-      <c r="D63" s="6"/>
-      <c r="E63" s="6"/>
+      <c r="A63" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D63" s="6">
+        <v>0</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="F63" t="s">
+        <v>167</v>
+      </c>
+      <c r="G63" s="6"/>
+      <c r="H63" s="6"/>
+      <c r="I63" s="6"/>
+      <c r="J63" s="6"/>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
-        <v>77</v>
+        <v>169</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>78</v>
+        <v>173</v>
       </c>
       <c r="D64" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F64" s="6" t="s">
-        <v>120</v>
+        <v>157</v>
+      </c>
+      <c r="F64" t="s">
+        <v>168</v>
       </c>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
@@ -2580,22 +2625,22 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
-        <v>77</v>
+        <v>170</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>78</v>
+        <v>174</v>
       </c>
       <c r="D65" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F65" s="6" t="s">
-        <v>79</v>
+        <v>157</v>
+      </c>
+      <c r="F65" t="s">
+        <v>164</v>
       </c>
       <c r="G65" s="6"/>
       <c r="H65" s="6"/>
@@ -2604,22 +2649,22 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
-        <v>77</v>
+        <v>170</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>78</v>
+        <v>174</v>
       </c>
       <c r="D66" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F66" s="6" t="s">
-        <v>80</v>
+        <v>157</v>
+      </c>
+      <c r="F66" t="s">
+        <v>165</v>
       </c>
       <c r="G66" s="6"/>
       <c r="H66" s="6"/>
@@ -2628,22 +2673,22 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
-        <v>81</v>
+        <v>170</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>82</v>
+        <v>174</v>
       </c>
       <c r="D67" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F67" s="6" t="s">
-        <v>83</v>
+        <v>157</v>
+      </c>
+      <c r="F67" t="s">
+        <v>166</v>
       </c>
       <c r="G67" s="6"/>
       <c r="H67" s="6"/>
@@ -2652,22 +2697,22 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="6" t="s">
-        <v>84</v>
+        <v>170</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>85</v>
+        <v>174</v>
       </c>
       <c r="D68" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F68" s="6" t="s">
-        <v>86</v>
+        <v>157</v>
+      </c>
+      <c r="F68" t="s">
+        <v>176</v>
       </c>
       <c r="G68" s="6"/>
       <c r="H68" s="6"/>
@@ -2676,85 +2721,64 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
-        <v>87</v>
+        <v>171</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>88</v>
+        <v>175</v>
       </c>
       <c r="D69" s="6">
         <v>0</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F69" s="6" t="s">
-        <v>89</v>
+        <v>157</v>
+      </c>
+      <c r="F69" t="s">
+        <v>162</v>
       </c>
       <c r="G69" s="6"/>
       <c r="H69" s="6"/>
       <c r="I69" s="6"/>
       <c r="J69" s="6"/>
     </row>
-    <row r="70" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
-        <v>90</v>
+        <v>171</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>91</v>
+        <v>175</v>
       </c>
       <c r="D70" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F70" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="G70" s="6"/>
-      <c r="H70" s="6"/>
-      <c r="I70" s="6"/>
-      <c r="J70" s="6"/>
+        <v>157</v>
+      </c>
+      <c r="F70" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A71" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B71" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="D71" s="6">
-        <v>0</v>
-      </c>
-      <c r="E71" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F71" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="G71" s="6"/>
-      <c r="H71" s="6"/>
-      <c r="I71" s="6"/>
-      <c r="J71" s="6"/>
+      <c r="A71" s="6"/>
+      <c r="B71" s="6"/>
+      <c r="C71" s="6"/>
+      <c r="D71" s="6"/>
+      <c r="E71" s="6"/>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="6" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="D72" s="6">
         <v>0</v>
@@ -2763,7 +2787,7 @@
         <v>41</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="G72" s="6"/>
       <c r="H72" s="6"/>
@@ -2771,98 +2795,290 @@
       <c r="J72" s="6"/>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
+      <c r="A73" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D73" s="6">
+        <v>1</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G73" s="6"/>
+      <c r="H73" s="6"/>
+      <c r="I73" s="6"/>
+      <c r="J73" s="6"/>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A74" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D74" s="6">
+        <v>2</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G74" s="6"/>
+      <c r="H74" s="6"/>
+      <c r="I74" s="6"/>
+      <c r="J74" s="6"/>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A75" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D75" s="6">
+        <v>0</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G75" s="6"/>
+      <c r="H75" s="6"/>
+      <c r="I75" s="6"/>
+      <c r="J75" s="6"/>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A76" s="6"/>
+      <c r="B76" s="6"/>
+      <c r="C76" s="6"/>
+      <c r="D76" s="6"/>
+      <c r="E76" s="6"/>
+      <c r="F76" s="6"/>
+      <c r="G76" s="6"/>
+      <c r="H76" s="6"/>
+      <c r="I76" s="6"/>
+      <c r="J76" s="6"/>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A77" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D77" s="6">
+        <v>0</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="G77" s="6"/>
+      <c r="H77" s="6"/>
+      <c r="I77" s="6"/>
+      <c r="J77" s="6"/>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A78" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D78" s="6">
+        <v>0</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="G78" s="6"/>
+      <c r="H78" s="6"/>
+      <c r="I78" s="6"/>
+      <c r="J78" s="6"/>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A79" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D79" s="6">
+        <v>0</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="G79" s="6"/>
+      <c r="H79" s="6"/>
+      <c r="I79" s="6"/>
+      <c r="J79" s="6"/>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A80" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D80" s="6">
+        <v>0</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G80" s="6"/>
+      <c r="H80" s="6"/>
+      <c r="I80" s="6"/>
+      <c r="J80" s="6"/>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A81" s="6"/>
+      <c r="B81" s="6"/>
+      <c r="C81" s="6"/>
+      <c r="D81" s="6"/>
+      <c r="E81" s="6"/>
+      <c r="F81" s="6"/>
+      <c r="G81" s="6"/>
+      <c r="H81" s="6"/>
+      <c r="I81" s="6"/>
+      <c r="J81" s="6"/>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
         <v>122</v>
       </c>
-      <c r="B73" s="6" t="s">
+      <c r="B82" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C82" t="s">
         <v>123</v>
       </c>
-      <c r="D73">
+      <c r="D82">
         <v>0</v>
       </c>
-      <c r="E73" t="s">
+      <c r="E82" t="s">
         <v>41</v>
       </c>
-      <c r="F73" t="s">
+      <c r="F82" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
         <v>122</v>
       </c>
-      <c r="B74" s="6" t="s">
+      <c r="B83" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C83" t="s">
         <v>123</v>
       </c>
-      <c r="D74">
+      <c r="D83">
         <v>1</v>
       </c>
-      <c r="E74" t="s">
+      <c r="E83" t="s">
         <v>124</v>
       </c>
-      <c r="F74" t="s">
+      <c r="F83" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
         <v>122</v>
       </c>
-      <c r="B75" s="6" t="s">
+      <c r="B84" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C75" t="s">
+      <c r="C84" t="s">
         <v>123</v>
       </c>
-      <c r="D75">
+      <c r="D84">
         <v>2</v>
       </c>
-      <c r="E75" t="s">
+      <c r="E84" t="s">
         <v>124</v>
       </c>
-      <c r="F75" t="s">
+      <c r="F84" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
         <v>122</v>
       </c>
-      <c r="B76" s="6" t="s">
+      <c r="B85" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C76" t="s">
+      <c r="C85" t="s">
         <v>123</v>
       </c>
-      <c r="D76">
+      <c r="D85">
         <v>3</v>
       </c>
-      <c r="E76" t="s">
+      <c r="E85" t="s">
         <v>41</v>
       </c>
-      <c r="F76" t="s">
+      <c r="F85" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A82" s="6"/>
-      <c r="B82" s="6"/>
-      <c r="C82" s="6"/>
-      <c r="D82" s="6"/>
-      <c r="E82" s="6"/>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A83" s="6"/>
-      <c r="B83" s="6"/>
-      <c r="C83" s="6"/>
-      <c r="D83" s="6"/>
-      <c r="E83" s="6"/>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A91" s="6"/>
+      <c r="B91" s="6"/>
+      <c r="C91" s="6"/>
+      <c r="D91" s="6"/>
+      <c r="E91" s="6"/>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A92" s="6"/>
+      <c r="B92" s="6"/>
+      <c r="C92" s="6"/>
+      <c r="D92" s="6"/>
+      <c r="E92" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>